<commit_message>
Add 40 emails scraped from CT fabricator websites
</commit_message>
<xml_diff>
--- a/public/fabricator-leads-CT.xlsx
+++ b/public/fabricator-leads-CT.xlsx
@@ -1201,7 +1201,7 @@
         <v>101 Wooster St Unit C Bethel CT 06801</v>
       </c>
       <c r="K23" t="str">
-        <v/>
+        <v>academymb@gmail.com</v>
       </c>
     </row>
     <row r="24">
@@ -1236,7 +1236,7 @@
         <v>155 Greenwood Ave Unit E102 Bethel CT 06801. Master fabricators.</v>
       </c>
       <c r="K24" t="str">
-        <v/>
+        <v>customerservice@jcsmarbleandgranite.com</v>
       </c>
     </row>
     <row r="25">
@@ -1271,7 +1271,7 @@
         <v>197 Ethan Allen Hwy Rte 7 Ridgefield CT 06877. Family-owned since 2008.</v>
       </c>
       <c r="K25" t="str">
-        <v/>
+        <v>veneziamarble@yahoo.com</v>
       </c>
     </row>
     <row r="26">
@@ -1306,7 +1306,7 @@
         <v>1106 Federal Rd Brookfield CT 06804. Also has Ridgefield location.</v>
       </c>
       <c r="K26" t="str">
-        <v/>
+        <v>sales@lapietramarble.com</v>
       </c>
     </row>
     <row r="27">
@@ -1341,7 +1341,7 @@
         <v>5 Danbury Rd New Milford CT 06776</v>
       </c>
       <c r="K27" t="str">
-        <v/>
+        <v>marblecreations@sbcglobal.net</v>
       </c>
     </row>
     <row r="28">
@@ -1376,7 +1376,7 @@
         <v>27 Pickett District Rd New Milford CT 06776</v>
       </c>
       <c r="K28" t="str">
-        <v/>
+        <v>jfgraniteandmarble@aol.com</v>
       </c>
     </row>
     <row r="29">
@@ -1446,7 +1446,7 @@
         <v>233 Asylum St Bridgeport CT 06610</v>
       </c>
       <c r="K30" t="str">
-        <v/>
+        <v>angelosmarble@yahoo.com</v>
       </c>
     </row>
     <row r="31">
@@ -1516,7 +1516,7 @@
         <v>1108 Railroad Ave Bridgeport CT 06605</v>
       </c>
       <c r="K32" t="str">
-        <v/>
+        <v>Daniel@thestoneworkshop.com</v>
       </c>
     </row>
     <row r="33">
@@ -1656,7 +1656,7 @@
         <v>261 River St Bridgeport CT 06604</v>
       </c>
       <c r="K36" t="str">
-        <v/>
+        <v>info@fairmarble.com</v>
       </c>
     </row>
     <row r="37">
@@ -1831,7 +1831,7 @@
         <v>365 Christian St Oxford CT 06478. Fabrication and installation.</v>
       </c>
       <c r="K41" t="str">
-        <v/>
+        <v>marbledesign02@gmail.com</v>
       </c>
     </row>
     <row r="42">
@@ -1866,7 +1866,7 @@
         <v>38 Triangle St Danbury CT 06810. Family-owned 19+ years.</v>
       </c>
       <c r="K42" t="str">
-        <v/>
+        <v>jrlgranitemarble@gmail.com</v>
       </c>
     </row>
     <row r="43">
@@ -1901,7 +1901,7 @@
         <v>92 North St Danbury CT 06810. In business since 1992.</v>
       </c>
       <c r="K43" t="str">
-        <v/>
+        <v>projects@stariancountertops.com</v>
       </c>
     </row>
     <row r="44">
@@ -1971,7 +1971,7 @@
         <v>420 Post Road West Westport CT 06880. 30+ years. 30000 sq ft stone slab selection and fabrication.</v>
       </c>
       <c r="K45" t="str">
-        <v/>
+        <v>dale@classicstones.com</v>
       </c>
     </row>
     <row r="46">
@@ -2041,7 +2041,7 @@
         <v>43 Huntington St Shelton CT 06484. Custom countertop and cabinet fabricator.</v>
       </c>
       <c r="K47" t="str">
-        <v/>
+        <v>info@diversifiedkitchensllc.com</v>
       </c>
     </row>
     <row r="48">
@@ -2076,7 +2076,7 @@
         <v>141 S Main St Beacon Falls CT 06403</v>
       </c>
       <c r="K48" t="str">
-        <v/>
+        <v>americanflagstones@att.net</v>
       </c>
     </row>
     <row r="49">
@@ -2111,7 +2111,7 @@
         <v>320 James St New Haven CT 06513. Family-owned since 1998.</v>
       </c>
       <c r="K49" t="str">
-        <v/>
+        <v>showroomcreative320@gmail.com</v>
       </c>
     </row>
     <row r="50">
@@ -2216,7 +2216,7 @@
         <v>23 Raccio Park Rd Hamden CT 06514</v>
       </c>
       <c r="K52" t="str">
-        <v/>
+        <v>sales@stonelabct.com</v>
       </c>
     </row>
     <row r="53">
@@ -2251,7 +2251,7 @@
         <v>55 Connair Rd Orange CT 06477</v>
       </c>
       <c r="K53" t="str">
-        <v/>
+        <v>info@thestonefactory.net</v>
       </c>
     </row>
     <row r="54">
@@ -2391,7 +2391,7 @@
         <v>201 Buckingham Ave Milford CT 06460</v>
       </c>
       <c r="K57" t="str">
-        <v/>
+        <v>easternmng@gmail.com</v>
       </c>
     </row>
     <row r="58">
@@ -2426,7 +2426,7 @@
         <v>80 Wampus Ln Milford CT 06460. 25+ years family-owned.</v>
       </c>
       <c r="K58" t="str">
-        <v/>
+        <v>stonegalaxy@yahoo.com</v>
       </c>
     </row>
     <row r="59">
@@ -2636,7 +2636,7 @@
         <v>43 Capital Dr Wallingford CT 06492</v>
       </c>
       <c r="K64" t="str">
-        <v/>
+        <v>sales@elevatedgranite.com</v>
       </c>
     </row>
     <row r="65">
@@ -3126,7 +3126,7 @@
         <v>239 Christian Ln Berlin CT 06037. Full fabrication facility. Serves Hartford and New Haven counties.</v>
       </c>
       <c r="K78" t="str">
-        <v/>
+        <v>sales@ambiancestone.com</v>
       </c>
     </row>
     <row r="79">
@@ -3196,7 +3196,7 @@
         <v>97 Airport Rd Hartford CT 06114. Family-owned since 1978.</v>
       </c>
       <c r="K80" t="str">
-        <v/>
+        <v>sabrina@pistrittomarble.com</v>
       </c>
     </row>
     <row r="81">
@@ -3231,7 +3231,7 @@
         <v>110 Airport Rd Hartford CT 06114</v>
       </c>
       <c r="K81" t="str">
-        <v/>
+        <v>sales@imagestonecenter.com</v>
       </c>
     </row>
     <row r="82">
@@ -3301,7 +3301,7 @@
         <v>60 Wooster St New Britain CT 06052. 10000 sq ft fabrication shop.</v>
       </c>
       <c r="K83" t="str">
-        <v/>
+        <v>info@stonevalleygranite.com</v>
       </c>
     </row>
     <row r="84">
@@ -3336,7 +3336,7 @@
         <v>8 Cody St West Hartford CT 06110</v>
       </c>
       <c r="K84" t="str">
-        <v/>
+        <v>negraniteandcabinets@gmail.com</v>
       </c>
     </row>
     <row r="85">
@@ -3371,7 +3371,7 @@
         <v>5 Albany Turnpike Unit B4 Canton CT</v>
       </c>
       <c r="K85" t="str">
-        <v/>
+        <v>info@glcstone.com</v>
       </c>
     </row>
     <row r="86">
@@ -3406,7 +3406,7 @@
         <v>1547 New Britain Ave Farmington CT 06032</v>
       </c>
       <c r="K86" t="str">
-        <v/>
+        <v>paul@ewgraniteandmarble.com</v>
       </c>
     </row>
     <row r="87">
@@ -3581,7 +3581,7 @@
         <v>4 Alcap Ridge Cromwell CT 06416. One of CT's largest countertop installers.</v>
       </c>
       <c r="K91" t="str">
-        <v/>
+        <v>nikki@cthardrock.com</v>
       </c>
     </row>
     <row r="92">
@@ -3791,7 +3791,7 @@
         <v>720 N Mountain Rd Newington CT 06111</v>
       </c>
       <c r="K97" t="str">
-        <v/>
+        <v>info@pioneerstoneworks.com</v>
       </c>
     </row>
     <row r="98">
@@ -3826,7 +3826,7 @@
         <v>43 Aircraft Rd Southington CT 06489</v>
       </c>
       <c r="K98" t="str">
-        <v/>
+        <v>info@gothicmg.com</v>
       </c>
     </row>
     <row r="99">
@@ -3896,7 +3896,7 @@
         <v>45 Ozick Dr Unit 1 Durham CT 06422. Artisan stone craftsmen est 1999.</v>
       </c>
       <c r="K100" t="str">
-        <v/>
+        <v>markjette@marbleandgranitecounters.com</v>
       </c>
     </row>
     <row r="101">
@@ -3931,7 +3931,7 @@
         <v>355 Farmington Ave Plainville CT 06062. 30+ years experience.</v>
       </c>
       <c r="K101" t="str">
-        <v/>
+        <v>eric@rosaniastonedesigns.com</v>
       </c>
     </row>
     <row r="102">
@@ -4001,7 +4001,7 @@
         <v>161 Woodford Ave Ste 48 Plainville CT 06062</v>
       </c>
       <c r="K103" t="str">
-        <v/>
+        <v>office@veronactgranitemarble.com</v>
       </c>
     </row>
     <row r="104">
@@ -4141,7 +4141,7 @@
         <v>313 Pleasant Valley Rd South Windsor CT 06074</v>
       </c>
       <c r="K107" t="str">
-        <v/>
+        <v>info@granitekitchenstudio.com</v>
       </c>
     </row>
     <row r="108">
@@ -4211,7 +4211,7 @@
         <v>59A King Spring Rd Windsor Locks CT 06096. Family-owned since 1999.</v>
       </c>
       <c r="K109" t="str">
-        <v/>
+        <v>info@draculamarbleandgranite.com</v>
       </c>
     </row>
     <row r="110">
@@ -4281,7 +4281,7 @@
         <v>450 Riverside Ave Bristol CT 06010. Family-run since 1972. Full fabrication shop.</v>
       </c>
       <c r="K111" t="str">
-        <v/>
+        <v>modern@moderncabinets.com</v>
       </c>
     </row>
     <row r="112">
@@ -4316,7 +4316,7 @@
         <v>33 River St Unit D Thomaston CT 06787. 35+ years experience.</v>
       </c>
       <c r="K112" t="str">
-        <v/>
+        <v>milestonegranite@att.net</v>
       </c>
     </row>
     <row r="113">
@@ -4456,7 +4456,7 @@
         <v>22 Vermont Dr Willimantic CT 06226. Premier soapstone fabricator New England.</v>
       </c>
       <c r="K116" t="str">
-        <v/>
+        <v>info@ctsoapstone.com</v>
       </c>
     </row>
     <row r="117">
@@ -4806,7 +4806,7 @@
         <v>120 East Haddam Rd Salem CT 06420. Custom granite countertops and stone surfaces.</v>
       </c>
       <c r="K126" t="str">
-        <v/>
+        <v>sales@gettygranite.com</v>
       </c>
     </row>
   </sheetData>

</xml_diff>